<commit_message>
Fix UAT_Tracker_Simple.xlsx - ensure all cells populated correctly
Co-authored-by: faiz1277 <161115614+faiz1277@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/UAT_Tracker_Simple.xlsx
+++ b/UAT_Tracker_Simple.xlsx
@@ -569,8 +569,8 @@
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
     <col width="28" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
@@ -648,11 +648,7 @@
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Check all fields are required</t>
-        </is>
-      </c>
+      <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr">
         <is>
           <t>07/08/2026</t>
@@ -696,7 +692,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Gated Access – Redirect</t>
+          <t>Gated Access - Redirect</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
@@ -848,11 +844,7 @@
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr"/>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>Should be accessible to all</t>
-        </is>
-      </c>
+      <c r="H9" s="3" t="inlineStr"/>
       <c r="I9" s="3" t="inlineStr">
         <is>
           <t>07/08/2026</t>
@@ -876,15 +868,11 @@
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Call &amp; put prices calculate correctly for given S, K, T, r, σ</t>
+          <t>Call &amp; put prices calculate correctly for given S, K, T, r, sigma</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Test with S=100, K=100, T=1, r=5%, σ=20%</t>
-        </is>
-      </c>
+      <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr">
         <is>
           <t>07/08/2026</t>
@@ -900,7 +888,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Greeks display (Delta, Gamma, Vega, Theta, Rho)</t>
+          <t>Greeks (Delta, Gamma, Vega, Theta, Rho)</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
@@ -1152,7 +1140,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Arithmetic average Asian pricing</t>
+          <t>Arithmetic average pricing</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr"/>
@@ -1180,7 +1168,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Geometric average Asian pricing</t>
+          <t>Geometric average pricing</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr"/>
@@ -1272,7 +1260,7 @@
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Capital loss scenario shown when knock-in barrier breached at maturity</t>
+          <t>Capital loss shown when knock-in barrier breached at maturity</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
@@ -1427,7 +1415,7 @@
     <row r="30" ht="22" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Fixed Income – Bonds</t>
+          <t>Fixed Income - Bonds</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1455,7 +1443,7 @@
     <row r="31" ht="22" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Fixed Income – Bonds</t>
+          <t>Fixed Income - Bonds</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1483,7 +1471,7 @@
     <row r="32" ht="22" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Fixed Income – Bonds</t>
+          <t>Fixed Income - Bonds</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1511,7 +1499,7 @@
     <row r="33" ht="22" customHeight="1">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Rates – Interest Rate Swap</t>
+          <t>Rates - Interest Rate Swap</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1539,7 +1527,7 @@
     <row r="34" ht="22" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Rates – Swaption</t>
+          <t>Rates - Swaption</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1567,7 +1555,7 @@
     <row r="35" ht="22" customHeight="1">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Rates – Forward Rate Agreement</t>
+          <t>Rates - FRA</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1595,7 +1583,7 @@
     <row r="36" ht="22" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Rates – Interest Rate Futures</t>
+          <t>Rates - IR Futures</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1707,7 +1695,7 @@
     <row r="40" ht="22" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Credit-Linked Note</t>
+          <t>CLN</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -1936,7 +1924,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Error handling – invalid inputs</t>
+          <t>Error handling - invalid inputs</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr"/>
@@ -1972,7 +1960,7 @@
       <c r="E49" s="3" t="inlineStr"/>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>Each product page loads within 3 seconds on standard connection</t>
+          <t>Each product page loads within 3 seconds</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr"/>
@@ -2010,20 +1998,20 @@
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>UAT Testing – Summary Dashboard</t>
+          <t>UAT Testing - Summary Dashboard</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-updated from "UAT Testing" sheet  |  Total test cases pre-loaded: 48</t>
+          <t>Auto-updated from 'UAT Testing' sheet  |  48 test cases pre-loaded</t>
         </is>
       </c>
     </row>
@@ -2062,7 +2050,7 @@
       <c r="C5" s="9" t="n"/>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>Fully functional – no issues</t>
+          <t>Fully functional</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2084,7 @@
       <c r="C7" s="9" t="n"/>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>Blocking – must fix before release</t>
+          <t>Blocking issues</t>
         </is>
       </c>
     </row>
@@ -2113,7 +2101,7 @@
       <c r="C8" s="9" t="n"/>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>Defect logged in bug tracker</t>
+          <t>Defect logged</t>
         </is>
       </c>
     </row>
@@ -2130,7 +2118,7 @@
       <c r="C9" s="9" t="n"/>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>Status cell left blank</t>
+          <t>Status blank</t>
         </is>
       </c>
     </row>
@@ -2150,7 +2138,7 @@
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>Pass Rate (Working only)</t>
+          <t>Pass Rate</t>
         </is>
       </c>
       <c r="B11" s="16">
@@ -2160,7 +2148,7 @@
       <c r="C11" s="9" t="n"/>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>Working ÷ Total Tests</t>
+          <t>Working / Total Tests</t>
         </is>
       </c>
     </row>

</xml_diff>